<commit_message>
Update Excel with Pez surname and app fixes
</commit_message>
<xml_diff>
--- a/Plantilla_Crecimiento_y_Maduracion.xlsx
+++ b/Plantilla_Crecimiento_y_Maduracion.xlsx
@@ -2,30 +2,34 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23801"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Daniel\Desktop\PRESENTACION CEPARD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dany\cloudestreamlit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E514DDF8-93BA-469C-8F21-BDF6F80AF1F4}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8F0171-D726-4D65-A091-3C7C4674DDE6}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F264843-BFA8-4D8F-9020-931CA3584421}"/>
+    <workbookView xWindow="3204" yWindow="2388" windowWidth="16488" windowHeight="9852" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="33">
+  <si>
+    <t>Nombre y Apellido</t>
+  </si>
+  <si>
+    <t>DNI</t>
+  </si>
+  <si>
+    <t>Sexo</t>
+  </si>
   <si>
     <t>Deporte</t>
   </si>
@@ -34,6 +38,9 @@
   </si>
   <si>
     <t>Fecha de Evaluacion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura de Pie </t>
   </si>
   <si>
     <t>Altura sentado</t>
@@ -48,25 +55,13 @@
     <t>Altura de la madre</t>
   </si>
   <si>
-    <t>Nombre y Apellido</t>
-  </si>
-  <si>
-    <t>Sexo</t>
-  </si>
-  <si>
-    <t>DNI</t>
-  </si>
-  <si>
-    <t>Sol Peso</t>
+    <t>Sol Pez</t>
   </si>
   <si>
     <t>F</t>
   </si>
   <si>
     <t>Talento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altura de Pie </t>
   </si>
   <si>
     <t>Ana Lopez</t>
@@ -111,6 +106,9 @@
     <t>Hugo Morales</t>
   </si>
   <si>
+    <t>Mateo Fantasia</t>
+  </si>
+  <si>
     <t>Tenis</t>
   </si>
   <si>
@@ -122,15 +120,12 @@
   <si>
     <t>Fútbol</t>
   </si>
-  <si>
-    <t>Mateo Fantasia</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -139,16 +134,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -160,7 +148,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -168,49 +156,21 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -233,44 +193,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -297,32 +257,14 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -349,24 +291,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -378,213 +302,226 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D23E8A2-5C4E-4CEB-BB7C-68680B17780E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="17.21875" customWidth="1"/>
-    <col min="2" max="3" width="16.109375" customWidth="1"/>
-    <col min="4" max="4" width="11.88671875" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" t="s">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K1" t="s">
-        <v>6</v>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>54035606</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="1">
+        <v>13</v>
+      </c>
+      <c r="E2">
         <v>41838</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2">
         <v>45703</v>
       </c>
       <c r="G2">
@@ -605,21 +542,21 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>54035606</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="1">
+        <v>13</v>
+      </c>
+      <c r="E3">
         <v>41838</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F3">
         <v>45772</v>
       </c>
       <c r="G3">
@@ -640,21 +577,21 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>54035606</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="1">
+        <v>13</v>
+      </c>
+      <c r="E4">
         <v>41838</v>
       </c>
-      <c r="F4" s="1">
+      <c r="F4">
         <v>45818</v>
       </c>
       <c r="G4">
@@ -675,21 +612,21 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5">
         <v>54035606</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="1">
+        <v>13</v>
+      </c>
+      <c r="E5">
         <v>41838</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5">
         <v>45889</v>
       </c>
       <c r="G5">
@@ -710,21 +647,21 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>54035606</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="1">
+        <v>13</v>
+      </c>
+      <c r="E6">
         <v>41838</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6">
         <v>45960</v>
       </c>
       <c r="G6">
@@ -745,21 +682,21 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7">
         <v>54035606</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="1">
+        <v>13</v>
+      </c>
+      <c r="E7">
         <v>41838</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7">
         <v>46006</v>
       </c>
       <c r="G7">
@@ -786,15 +723,15 @@
         <v>10101001</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8">
         <v>41039</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8">
         <v>45703</v>
       </c>
       <c r="G8">
@@ -821,15 +758,15 @@
         <v>10101001</v>
       </c>
       <c r="C9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D9" t="s">
         <v>15</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9">
         <v>41039</v>
       </c>
-      <c r="F9" s="1">
+      <c r="F9">
         <v>45772</v>
       </c>
       <c r="G9">
@@ -856,15 +793,15 @@
         <v>10101001</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10">
         <v>41039</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10">
         <v>45818</v>
       </c>
       <c r="G10">
@@ -891,15 +828,15 @@
         <v>10101001</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11">
         <v>41039</v>
       </c>
-      <c r="F11" s="1">
+      <c r="F11">
         <v>45889</v>
       </c>
       <c r="G11">
@@ -926,15 +863,15 @@
         <v>10101001</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12">
         <v>41039</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12">
         <v>45960</v>
       </c>
       <c r="G12">
@@ -961,15 +898,15 @@
         <v>10101001</v>
       </c>
       <c r="C13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D13" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13">
         <v>41039</v>
       </c>
-      <c r="F13" s="1">
+      <c r="F13">
         <v>46006</v>
       </c>
       <c r="G13">
@@ -996,15 +933,15 @@
         <v>10101002</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D14" t="s">
         <v>17</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14">
         <v>40777</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14">
         <v>45703</v>
       </c>
       <c r="G14">
@@ -1031,15 +968,15 @@
         <v>10101002</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15">
         <v>40777</v>
       </c>
-      <c r="F15" s="1">
+      <c r="F15">
         <v>45772</v>
       </c>
       <c r="G15">
@@ -1066,15 +1003,15 @@
         <v>10101002</v>
       </c>
       <c r="C16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D16" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16">
         <v>40777</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16">
         <v>45818</v>
       </c>
       <c r="G16">
@@ -1101,15 +1038,15 @@
         <v>10101002</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D17" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17">
         <v>40777</v>
       </c>
-      <c r="F17" s="1">
+      <c r="F17">
         <v>45889</v>
       </c>
       <c r="G17">
@@ -1136,15 +1073,15 @@
         <v>10101002</v>
       </c>
       <c r="C18" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D18" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18">
         <v>40777</v>
       </c>
-      <c r="F18" s="1">
+      <c r="F18">
         <v>45960</v>
       </c>
       <c r="G18">
@@ -1171,15 +1108,15 @@
         <v>10101002</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D19" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19">
         <v>40777</v>
       </c>
-      <c r="F19" s="1">
+      <c r="F19">
         <v>46006</v>
       </c>
       <c r="G19">
@@ -1206,15 +1143,15 @@
         <v>10101003</v>
       </c>
       <c r="C20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D20" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20">
         <v>41320</v>
       </c>
-      <c r="F20" s="1">
+      <c r="F20">
         <v>45703</v>
       </c>
       <c r="G20">
@@ -1241,15 +1178,15 @@
         <v>10101003</v>
       </c>
       <c r="C21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D21" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21">
         <v>41320</v>
       </c>
-      <c r="F21" s="1">
+      <c r="F21">
         <v>45772</v>
       </c>
       <c r="G21">
@@ -1276,15 +1213,15 @@
         <v>10101003</v>
       </c>
       <c r="C22" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D22" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="1">
+      <c r="E22">
         <v>41320</v>
       </c>
-      <c r="F22" s="1">
+      <c r="F22">
         <v>45818</v>
       </c>
       <c r="G22">
@@ -1311,15 +1248,15 @@
         <v>10101003</v>
       </c>
       <c r="C23" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D23" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23">
         <v>41320</v>
       </c>
-      <c r="F23" s="1">
+      <c r="F23">
         <v>45889</v>
       </c>
       <c r="G23">
@@ -1346,15 +1283,15 @@
         <v>10101003</v>
       </c>
       <c r="C24" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="1">
+      <c r="E24">
         <v>41320</v>
       </c>
-      <c r="F24" s="1">
+      <c r="F24">
         <v>45960</v>
       </c>
       <c r="G24">
@@ -1381,15 +1318,15 @@
         <v>10101003</v>
       </c>
       <c r="C25" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D25" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="1">
+      <c r="E25">
         <v>41320</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25">
         <v>46006</v>
       </c>
       <c r="G25">
@@ -1416,15 +1353,15 @@
         <v>10101004</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D26" t="s">
         <v>21</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26">
         <v>40571</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26">
         <v>45703</v>
       </c>
       <c r="G26">
@@ -1451,15 +1388,15 @@
         <v>10101004</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D27" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="1">
+      <c r="E27">
         <v>40571</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F27">
         <v>45772</v>
       </c>
       <c r="G27">
@@ -1486,15 +1423,15 @@
         <v>10101004</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D28" t="s">
         <v>21</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28">
         <v>40571</v>
       </c>
-      <c r="F28" s="1">
+      <c r="F28">
         <v>45818</v>
       </c>
       <c r="G28">
@@ -1521,15 +1458,15 @@
         <v>10101004</v>
       </c>
       <c r="C29" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D29" t="s">
         <v>21</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29">
         <v>40571</v>
       </c>
-      <c r="F29" s="1">
+      <c r="F29">
         <v>45889</v>
       </c>
       <c r="G29">
@@ -1556,15 +1493,15 @@
         <v>10101004</v>
       </c>
       <c r="C30" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D30" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30">
         <v>40571</v>
       </c>
-      <c r="F30" s="1">
+      <c r="F30">
         <v>45960</v>
       </c>
       <c r="G30">
@@ -1591,15 +1528,15 @@
         <v>10101004</v>
       </c>
       <c r="C31" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D31" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="1">
+      <c r="E31">
         <v>40571</v>
       </c>
-      <c r="F31" s="1">
+      <c r="F31">
         <v>46006</v>
       </c>
       <c r="G31">
@@ -1626,15 +1563,15 @@
         <v>10101005</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D32" t="s">
         <v>15</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E32">
         <v>41548</v>
       </c>
-      <c r="F32" s="1">
+      <c r="F32">
         <v>45703</v>
       </c>
       <c r="G32">
@@ -1661,15 +1598,15 @@
         <v>10101005</v>
       </c>
       <c r="C33" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D33" t="s">
         <v>15</v>
       </c>
-      <c r="E33" s="1">
+      <c r="E33">
         <v>41548</v>
       </c>
-      <c r="F33" s="1">
+      <c r="F33">
         <v>45772</v>
       </c>
       <c r="G33">
@@ -1696,15 +1633,15 @@
         <v>10101005</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D34" t="s">
         <v>15</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34">
         <v>41548</v>
       </c>
-      <c r="F34" s="1">
+      <c r="F34">
         <v>45818</v>
       </c>
       <c r="G34">
@@ -1731,15 +1668,15 @@
         <v>10101005</v>
       </c>
       <c r="C35" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D35" t="s">
         <v>15</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35">
         <v>41548</v>
       </c>
-      <c r="F35" s="1">
+      <c r="F35">
         <v>45889</v>
       </c>
       <c r="G35">
@@ -1766,15 +1703,15 @@
         <v>10101005</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D36" t="s">
         <v>15</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36">
         <v>41548</v>
       </c>
-      <c r="F36" s="1">
+      <c r="F36">
         <v>45960</v>
       </c>
       <c r="G36">
@@ -1801,15 +1738,15 @@
         <v>10101005</v>
       </c>
       <c r="C37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D37" t="s">
         <v>15</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37">
         <v>41548</v>
       </c>
-      <c r="F37" s="1">
+      <c r="F37">
         <v>46006</v>
       </c>
       <c r="G37">
@@ -1841,10 +1778,10 @@
       <c r="D38" t="s">
         <v>19</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38">
         <v>40867</v>
       </c>
-      <c r="F38" s="1">
+      <c r="F38">
         <v>45703</v>
       </c>
       <c r="G38">
@@ -1876,10 +1813,10 @@
       <c r="D39" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39">
         <v>40867</v>
       </c>
-      <c r="F39" s="1">
+      <c r="F39">
         <v>45772</v>
       </c>
       <c r="G39">
@@ -1911,10 +1848,10 @@
       <c r="D40" t="s">
         <v>19</v>
       </c>
-      <c r="E40" s="1">
+      <c r="E40">
         <v>40867</v>
       </c>
-      <c r="F40" s="1">
+      <c r="F40">
         <v>45818</v>
       </c>
       <c r="G40">
@@ -1946,10 +1883,10 @@
       <c r="D41" t="s">
         <v>19</v>
       </c>
-      <c r="E41" s="1">
+      <c r="E41">
         <v>40867</v>
       </c>
-      <c r="F41" s="1">
+      <c r="F41">
         <v>45889</v>
       </c>
       <c r="G41">
@@ -1981,10 +1918,10 @@
       <c r="D42" t="s">
         <v>19</v>
       </c>
-      <c r="E42" s="1">
+      <c r="E42">
         <v>40867</v>
       </c>
-      <c r="F42" s="1">
+      <c r="F42">
         <v>45960</v>
       </c>
       <c r="G42">
@@ -2016,10 +1953,10 @@
       <c r="D43" t="s">
         <v>19</v>
       </c>
-      <c r="E43" s="1">
+      <c r="E43">
         <v>40867</v>
       </c>
-      <c r="F43" s="1">
+      <c r="F43">
         <v>46006</v>
       </c>
       <c r="G43">
@@ -2051,10 +1988,10 @@
       <c r="D44" t="s">
         <v>21</v>
       </c>
-      <c r="E44" s="1">
+      <c r="E44">
         <v>40426</v>
       </c>
-      <c r="F44" s="1">
+      <c r="F44">
         <v>45703</v>
       </c>
       <c r="G44">
@@ -2086,10 +2023,10 @@
       <c r="D45" t="s">
         <v>21</v>
       </c>
-      <c r="E45" s="1">
+      <c r="E45">
         <v>40426</v>
       </c>
-      <c r="F45" s="1">
+      <c r="F45">
         <v>45772</v>
       </c>
       <c r="G45">
@@ -2121,10 +2058,10 @@
       <c r="D46" t="s">
         <v>21</v>
       </c>
-      <c r="E46" s="1">
+      <c r="E46">
         <v>40426</v>
       </c>
-      <c r="F46" s="1">
+      <c r="F46">
         <v>45818</v>
       </c>
       <c r="G46">
@@ -2156,10 +2093,10 @@
       <c r="D47" t="s">
         <v>21</v>
       </c>
-      <c r="E47" s="1">
+      <c r="E47">
         <v>40426</v>
       </c>
-      <c r="F47" s="1">
+      <c r="F47">
         <v>45889</v>
       </c>
       <c r="G47">
@@ -2191,10 +2128,10 @@
       <c r="D48" t="s">
         <v>21</v>
       </c>
-      <c r="E48" s="1">
+      <c r="E48">
         <v>40426</v>
       </c>
-      <c r="F48" s="1">
+      <c r="F48">
         <v>45960</v>
       </c>
       <c r="G48">
@@ -2226,10 +2163,10 @@
       <c r="D49" t="s">
         <v>21</v>
       </c>
-      <c r="E49" s="1">
+      <c r="E49">
         <v>40426</v>
       </c>
-      <c r="F49" s="1">
+      <c r="F49">
         <v>46006</v>
       </c>
       <c r="G49">
@@ -2261,10 +2198,10 @@
       <c r="D50" t="s">
         <v>17</v>
       </c>
-      <c r="E50" s="1">
+      <c r="E50">
         <v>41102</v>
       </c>
-      <c r="F50" s="1">
+      <c r="F50">
         <v>45703</v>
       </c>
       <c r="G50">
@@ -2296,10 +2233,10 @@
       <c r="D51" t="s">
         <v>17</v>
       </c>
-      <c r="E51" s="1">
+      <c r="E51">
         <v>41102</v>
       </c>
-      <c r="F51" s="1">
+      <c r="F51">
         <v>45772</v>
       </c>
       <c r="G51">
@@ -2331,10 +2268,10 @@
       <c r="D52" t="s">
         <v>17</v>
       </c>
-      <c r="E52" s="1">
+      <c r="E52">
         <v>41102</v>
       </c>
-      <c r="F52" s="1">
+      <c r="F52">
         <v>45818</v>
       </c>
       <c r="G52">
@@ -2366,10 +2303,10 @@
       <c r="D53" t="s">
         <v>17</v>
       </c>
-      <c r="E53" s="1">
+      <c r="E53">
         <v>41102</v>
       </c>
-      <c r="F53" s="1">
+      <c r="F53">
         <v>45889</v>
       </c>
       <c r="G53">
@@ -2401,10 +2338,10 @@
       <c r="D54" t="s">
         <v>17</v>
       </c>
-      <c r="E54" s="1">
+      <c r="E54">
         <v>41102</v>
       </c>
-      <c r="F54" s="1">
+      <c r="F54">
         <v>45960</v>
       </c>
       <c r="G54">
@@ -2436,10 +2373,10 @@
       <c r="D55" t="s">
         <v>17</v>
       </c>
-      <c r="E55" s="1">
+      <c r="E55">
         <v>41102</v>
       </c>
-      <c r="F55" s="1">
+      <c r="F55">
         <v>46006</v>
       </c>
       <c r="G55">
@@ -2471,10 +2408,10 @@
       <c r="D56" t="s">
         <v>19</v>
       </c>
-      <c r="E56" s="1">
+      <c r="E56">
         <v>41358</v>
       </c>
-      <c r="F56" s="1">
+      <c r="F56">
         <v>45703</v>
       </c>
       <c r="G56">
@@ -2506,10 +2443,10 @@
       <c r="D57" t="s">
         <v>19</v>
       </c>
-      <c r="E57" s="1">
+      <c r="E57">
         <v>41358</v>
       </c>
-      <c r="F57" s="1">
+      <c r="F57">
         <v>45772</v>
       </c>
       <c r="G57">
@@ -2541,10 +2478,10 @@
       <c r="D58" t="s">
         <v>19</v>
       </c>
-      <c r="E58" s="1">
+      <c r="E58">
         <v>41358</v>
       </c>
-      <c r="F58" s="1">
+      <c r="F58">
         <v>45818</v>
       </c>
       <c r="G58">
@@ -2576,10 +2513,10 @@
       <c r="D59" t="s">
         <v>19</v>
       </c>
-      <c r="E59" s="1">
+      <c r="E59">
         <v>41358</v>
       </c>
-      <c r="F59" s="1">
+      <c r="F59">
         <v>45889</v>
       </c>
       <c r="G59">
@@ -2611,10 +2548,10 @@
       <c r="D60" t="s">
         <v>19</v>
       </c>
-      <c r="E60" s="1">
+      <c r="E60">
         <v>41358</v>
       </c>
-      <c r="F60" s="1">
+      <c r="F60">
         <v>45960</v>
       </c>
       <c r="G60">
@@ -2633,8 +2570,8 @@
         <v>163</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="5" t="s">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
         <v>27</v>
       </c>
       <c r="B61">
@@ -2646,10 +2583,10 @@
       <c r="D61" t="s">
         <v>19</v>
       </c>
-      <c r="E61" s="1">
+      <c r="E61">
         <v>41358</v>
       </c>
-      <c r="F61" s="1">
+      <c r="F61">
         <v>46006</v>
       </c>
       <c r="G61">
@@ -2668,637 +2605,637 @@
         <v>163</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="6" t="s">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>28</v>
+      </c>
+      <c r="B62">
+        <v>101</v>
+      </c>
+      <c r="C62" t="s">
+        <v>24</v>
+      </c>
+      <c r="D62" t="s">
+        <v>29</v>
+      </c>
+      <c r="E62">
+        <v>41044</v>
+      </c>
+      <c r="F62">
+        <v>45698</v>
+      </c>
+      <c r="G62">
+        <v>152</v>
+      </c>
+      <c r="H62">
+        <v>78.5</v>
+      </c>
+      <c r="I62">
+        <v>42</v>
+      </c>
+      <c r="J62">
+        <v>180</v>
+      </c>
+      <c r="K62">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>28</v>
+      </c>
+      <c r="B63">
+        <v>101</v>
+      </c>
+      <c r="C63" t="s">
+        <v>24</v>
+      </c>
+      <c r="D63" t="s">
+        <v>29</v>
+      </c>
+      <c r="E63">
+        <v>41044</v>
+      </c>
+      <c r="F63">
+        <v>45762</v>
+      </c>
+      <c r="G63">
+        <v>153.19999999999999</v>
+      </c>
+      <c r="H63">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="I63">
+        <v>42.8</v>
+      </c>
+      <c r="J63">
+        <v>180</v>
+      </c>
+      <c r="K63">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>28</v>
+      </c>
+      <c r="B64">
+        <v>101</v>
+      </c>
+      <c r="C64" t="s">
+        <v>24</v>
+      </c>
+      <c r="D64" t="s">
+        <v>29</v>
+      </c>
+      <c r="E64">
+        <v>41044</v>
+      </c>
+      <c r="F64">
+        <v>45828</v>
+      </c>
+      <c r="G64">
+        <v>154.5</v>
+      </c>
+      <c r="H64">
+        <v>79.8</v>
+      </c>
+      <c r="I64">
+        <v>43.5</v>
+      </c>
+      <c r="J64">
+        <v>180</v>
+      </c>
+      <c r="K64">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>28</v>
+      </c>
+      <c r="B65">
+        <v>101</v>
+      </c>
+      <c r="C65" t="s">
+        <v>24</v>
+      </c>
+      <c r="D65" t="s">
+        <v>29</v>
+      </c>
+      <c r="E65">
+        <v>41044</v>
+      </c>
+      <c r="F65">
+        <v>45894</v>
+      </c>
+      <c r="G65">
+        <v>155.80000000000001</v>
+      </c>
+      <c r="H65">
+        <v>80.400000000000006</v>
+      </c>
+      <c r="I65">
+        <v>44.2</v>
+      </c>
+      <c r="J65">
+        <v>180</v>
+      </c>
+      <c r="K65">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>28</v>
+      </c>
+      <c r="B66">
+        <v>101</v>
+      </c>
+      <c r="C66" t="s">
+        <v>24</v>
+      </c>
+      <c r="D66" t="s">
+        <v>29</v>
+      </c>
+      <c r="E66">
+        <v>41044</v>
+      </c>
+      <c r="F66">
+        <v>45960</v>
+      </c>
+      <c r="G66">
+        <v>157.1</v>
+      </c>
+      <c r="H66">
+        <v>81.099999999999994</v>
+      </c>
+      <c r="I66">
+        <v>45</v>
+      </c>
+      <c r="J66">
+        <v>180</v>
+      </c>
+      <c r="K66">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>28</v>
+      </c>
+      <c r="B67">
+        <v>101</v>
+      </c>
+      <c r="C67" t="s">
+        <v>24</v>
+      </c>
+      <c r="D67" t="s">
+        <v>29</v>
+      </c>
+      <c r="E67">
+        <v>41044</v>
+      </c>
+      <c r="F67">
+        <v>46006</v>
+      </c>
+      <c r="G67">
+        <v>158.4</v>
+      </c>
+      <c r="H67">
+        <v>81.7</v>
+      </c>
+      <c r="I67">
+        <v>45.8</v>
+      </c>
+      <c r="J67">
+        <v>180</v>
+      </c>
+      <c r="K67">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>30</v>
+      </c>
+      <c r="B68">
+        <v>102</v>
+      </c>
+      <c r="C68" t="s">
+        <v>12</v>
+      </c>
+      <c r="D68" t="s">
+        <v>17</v>
+      </c>
+      <c r="E68">
+        <v>41508</v>
+      </c>
+      <c r="F68">
+        <v>45698</v>
+      </c>
+      <c r="G68">
+        <v>148</v>
+      </c>
+      <c r="H68">
+        <v>75</v>
+      </c>
+      <c r="I68">
+        <v>38</v>
+      </c>
+      <c r="J68">
+        <v>175</v>
+      </c>
+      <c r="K68">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>30</v>
+      </c>
+      <c r="B69">
+        <v>102</v>
+      </c>
+      <c r="C69" t="s">
+        <v>12</v>
+      </c>
+      <c r="D69" t="s">
+        <v>17</v>
+      </c>
+      <c r="E69">
+        <v>41508</v>
+      </c>
+      <c r="F69">
+        <v>45762</v>
+      </c>
+      <c r="G69">
+        <v>149.5</v>
+      </c>
+      <c r="H69">
+        <v>75.8</v>
+      </c>
+      <c r="I69">
+        <v>39.1</v>
+      </c>
+      <c r="J69">
+        <v>175</v>
+      </c>
+      <c r="K69">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>30</v>
+      </c>
+      <c r="B70">
+        <v>102</v>
+      </c>
+      <c r="C70" t="s">
+        <v>12</v>
+      </c>
+      <c r="D70" t="s">
+        <v>17</v>
+      </c>
+      <c r="E70">
+        <v>41508</v>
+      </c>
+      <c r="F70">
+        <v>45828</v>
+      </c>
+      <c r="G70">
+        <v>151</v>
+      </c>
+      <c r="H70">
+        <v>76.5</v>
+      </c>
+      <c r="I70">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="J70">
+        <v>175</v>
+      </c>
+      <c r="K70">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>30</v>
+      </c>
+      <c r="B71">
+        <v>102</v>
+      </c>
+      <c r="C71" t="s">
+        <v>12</v>
+      </c>
+      <c r="D71" t="s">
+        <v>17</v>
+      </c>
+      <c r="E71">
+        <v>41508</v>
+      </c>
+      <c r="F71">
+        <v>45894</v>
+      </c>
+      <c r="G71">
+        <v>152.4</v>
+      </c>
+      <c r="H71">
+        <v>77.3</v>
+      </c>
+      <c r="I71">
+        <v>41.3</v>
+      </c>
+      <c r="J71">
+        <v>175</v>
+      </c>
+      <c r="K71">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>30</v>
+      </c>
+      <c r="B72">
+        <v>102</v>
+      </c>
+      <c r="C72" t="s">
+        <v>12</v>
+      </c>
+      <c r="D72" t="s">
+        <v>17</v>
+      </c>
+      <c r="E72">
+        <v>41508</v>
+      </c>
+      <c r="F72">
+        <v>45960</v>
+      </c>
+      <c r="G72">
+        <v>153.80000000000001</v>
+      </c>
+      <c r="H72">
+        <v>78.099999999999994</v>
+      </c>
+      <c r="I72">
+        <v>42.4</v>
+      </c>
+      <c r="J72">
+        <v>175</v>
+      </c>
+      <c r="K72">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>30</v>
+      </c>
+      <c r="B73">
+        <v>102</v>
+      </c>
+      <c r="C73" t="s">
+        <v>12</v>
+      </c>
+      <c r="D73" t="s">
+        <v>17</v>
+      </c>
+      <c r="E73">
+        <v>41508</v>
+      </c>
+      <c r="F73">
+        <v>46006</v>
+      </c>
+      <c r="G73">
+        <v>155.19999999999999</v>
+      </c>
+      <c r="H73">
+        <v>78.900000000000006</v>
+      </c>
+      <c r="I73">
+        <v>43.5</v>
+      </c>
+      <c r="J73">
+        <v>175</v>
+      </c>
+      <c r="K73">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>31</v>
+      </c>
+      <c r="B74">
+        <v>103</v>
+      </c>
+      <c r="C74" t="s">
+        <v>24</v>
+      </c>
+      <c r="D74" t="s">
         <v>32</v>
       </c>
-      <c r="B62" s="3">
-        <v>101</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E62" s="4">
-        <v>41044</v>
-      </c>
-      <c r="F62" s="4">
+      <c r="E74">
+        <v>40553</v>
+      </c>
+      <c r="F74">
         <v>45698</v>
       </c>
-      <c r="G62" s="3">
-        <v>152</v>
-      </c>
-      <c r="H62" s="3">
-        <v>78.5</v>
-      </c>
-      <c r="I62" s="3">
-        <v>42</v>
-      </c>
-      <c r="J62" s="3">
-        <v>180</v>
-      </c>
-      <c r="K62" s="3">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="6" t="s">
+      <c r="G74">
+        <v>162</v>
+      </c>
+      <c r="H74">
+        <v>83</v>
+      </c>
+      <c r="I74">
+        <v>52</v>
+      </c>
+      <c r="J74">
+        <v>182</v>
+      </c>
+      <c r="K74">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>31</v>
+      </c>
+      <c r="B75">
+        <v>103</v>
+      </c>
+      <c r="C75" t="s">
+        <v>24</v>
+      </c>
+      <c r="D75" t="s">
         <v>32</v>
       </c>
-      <c r="B63" s="3">
-        <v>101</v>
-      </c>
-      <c r="C63" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D63" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E63" s="4">
-        <v>41044</v>
-      </c>
-      <c r="F63" s="4">
+      <c r="E75">
+        <v>40553</v>
+      </c>
+      <c r="F75">
         <v>45762</v>
       </c>
-      <c r="G63" s="3">
-        <v>153.19999999999999</v>
-      </c>
-      <c r="H63" s="3">
-        <v>79.099999999999994</v>
-      </c>
-      <c r="I63" s="3">
-        <v>42.8</v>
-      </c>
-      <c r="J63" s="3">
-        <v>180</v>
-      </c>
-      <c r="K63" s="3">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="6" t="s">
+      <c r="G75">
+        <v>162.80000000000001</v>
+      </c>
+      <c r="H75">
+        <v>83.4</v>
+      </c>
+      <c r="I75">
+        <v>52.7</v>
+      </c>
+      <c r="J75">
+        <v>182</v>
+      </c>
+      <c r="K75">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>31</v>
+      </c>
+      <c r="B76">
+        <v>103</v>
+      </c>
+      <c r="C76" t="s">
+        <v>24</v>
+      </c>
+      <c r="D76" t="s">
         <v>32</v>
       </c>
-      <c r="B64" s="3">
-        <v>101</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E64" s="4">
-        <v>41044</v>
-      </c>
-      <c r="F64" s="4">
+      <c r="E76">
+        <v>40553</v>
+      </c>
+      <c r="F76">
         <v>45828</v>
       </c>
-      <c r="G64" s="3">
-        <v>154.5</v>
-      </c>
-      <c r="H64" s="3">
-        <v>79.8</v>
-      </c>
-      <c r="I64" s="3">
-        <v>43.5</v>
-      </c>
-      <c r="J64" s="3">
-        <v>180</v>
-      </c>
-      <c r="K64" s="3">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="6" t="s">
+      <c r="G76">
+        <v>163.6</v>
+      </c>
+      <c r="H76">
+        <v>83.8</v>
+      </c>
+      <c r="I76">
+        <v>53.4</v>
+      </c>
+      <c r="J76">
+        <v>182</v>
+      </c>
+      <c r="K76">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>31</v>
+      </c>
+      <c r="B77">
+        <v>103</v>
+      </c>
+      <c r="C77" t="s">
+        <v>24</v>
+      </c>
+      <c r="D77" t="s">
         <v>32</v>
       </c>
-      <c r="B65" s="3">
-        <v>101</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D65" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E65" s="4">
-        <v>41044</v>
-      </c>
-      <c r="F65" s="4">
+      <c r="E77">
+        <v>40553</v>
+      </c>
+      <c r="F77">
         <v>45894</v>
       </c>
-      <c r="G65" s="3">
-        <v>155.80000000000001</v>
-      </c>
-      <c r="H65" s="3">
-        <v>80.400000000000006</v>
-      </c>
-      <c r="I65" s="3">
-        <v>44.2</v>
-      </c>
-      <c r="J65" s="3">
-        <v>180</v>
-      </c>
-      <c r="K65" s="3">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="6" t="s">
+      <c r="G77">
+        <v>164.4</v>
+      </c>
+      <c r="H77">
+        <v>84.2</v>
+      </c>
+      <c r="I77">
+        <v>54.1</v>
+      </c>
+      <c r="J77">
+        <v>182</v>
+      </c>
+      <c r="K77">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>31</v>
+      </c>
+      <c r="B78">
+        <v>103</v>
+      </c>
+      <c r="C78" t="s">
+        <v>24</v>
+      </c>
+      <c r="D78" t="s">
         <v>32</v>
       </c>
-      <c r="B66" s="3">
-        <v>101</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E66" s="4">
-        <v>41044</v>
-      </c>
-      <c r="F66" s="4">
+      <c r="E78">
+        <v>40553</v>
+      </c>
+      <c r="F78">
         <v>45960</v>
       </c>
-      <c r="G66" s="3">
-        <v>157.1</v>
-      </c>
-      <c r="H66" s="3">
-        <v>81.099999999999994</v>
-      </c>
-      <c r="I66" s="3">
-        <v>45</v>
-      </c>
-      <c r="J66" s="3">
-        <v>180</v>
-      </c>
-      <c r="K66" s="3">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="6" t="s">
+      <c r="G78">
+        <v>165.2</v>
+      </c>
+      <c r="H78">
+        <v>84.6</v>
+      </c>
+      <c r="I78">
+        <v>54.8</v>
+      </c>
+      <c r="J78">
+        <v>182</v>
+      </c>
+      <c r="K78">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>31</v>
+      </c>
+      <c r="B79">
+        <v>103</v>
+      </c>
+      <c r="C79" t="s">
+        <v>24</v>
+      </c>
+      <c r="D79" t="s">
         <v>32</v>
       </c>
-      <c r="B67" s="3">
-        <v>101</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E67" s="4">
-        <v>41044</v>
-      </c>
-      <c r="F67" s="4">
+      <c r="E79">
+        <v>40553</v>
+      </c>
+      <c r="F79">
         <v>46006</v>
       </c>
-      <c r="G67" s="3">
-        <v>158.4</v>
-      </c>
-      <c r="H67" s="3">
-        <v>81.7</v>
-      </c>
-      <c r="I67" s="3">
-        <v>45.8</v>
-      </c>
-      <c r="J67" s="3">
-        <v>180</v>
-      </c>
-      <c r="K67" s="3">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B68" s="3">
-        <v>102</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E68" s="4">
-        <v>41508</v>
-      </c>
-      <c r="F68" s="4">
-        <v>45698</v>
-      </c>
-      <c r="G68" s="3">
-        <v>148</v>
-      </c>
-      <c r="H68" s="3">
-        <v>75</v>
-      </c>
-      <c r="I68" s="3">
-        <v>38</v>
-      </c>
-      <c r="J68" s="3">
-        <v>175</v>
-      </c>
-      <c r="K68" s="3">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B69" s="3">
-        <v>102</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E69" s="4">
-        <v>41508</v>
-      </c>
-      <c r="F69" s="4">
-        <v>45762</v>
-      </c>
-      <c r="G69" s="3">
-        <v>149.5</v>
-      </c>
-      <c r="H69" s="3">
-        <v>75.8</v>
-      </c>
-      <c r="I69" s="3">
-        <v>39.1</v>
-      </c>
-      <c r="J69" s="3">
-        <v>175</v>
-      </c>
-      <c r="K69" s="3">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B70" s="3">
-        <v>102</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E70" s="4">
-        <v>41508</v>
-      </c>
-      <c r="F70" s="4">
-        <v>45828</v>
-      </c>
-      <c r="G70" s="3">
-        <v>151</v>
-      </c>
-      <c r="H70" s="3">
-        <v>76.5</v>
-      </c>
-      <c r="I70" s="3">
-        <v>40.200000000000003</v>
-      </c>
-      <c r="J70" s="3">
-        <v>175</v>
-      </c>
-      <c r="K70" s="3">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B71" s="3">
-        <v>102</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E71" s="4">
-        <v>41508</v>
-      </c>
-      <c r="F71" s="4">
-        <v>45894</v>
-      </c>
-      <c r="G71" s="3">
-        <v>152.4</v>
-      </c>
-      <c r="H71" s="3">
-        <v>77.3</v>
-      </c>
-      <c r="I71" s="3">
-        <v>41.3</v>
-      </c>
-      <c r="J71" s="3">
-        <v>175</v>
-      </c>
-      <c r="K71" s="3">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B72" s="3">
-        <v>102</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E72" s="4">
-        <v>41508</v>
-      </c>
-      <c r="F72" s="4">
-        <v>45960</v>
-      </c>
-      <c r="G72" s="3">
-        <v>153.80000000000001</v>
-      </c>
-      <c r="H72" s="3">
-        <v>78.099999999999994</v>
-      </c>
-      <c r="I72" s="3">
-        <v>42.4</v>
-      </c>
-      <c r="J72" s="3">
-        <v>175</v>
-      </c>
-      <c r="K72" s="3">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B73" s="3">
-        <v>102</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D73" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E73" s="4">
-        <v>41508</v>
-      </c>
-      <c r="F73" s="4">
-        <v>46006</v>
-      </c>
-      <c r="G73" s="3">
-        <v>155.19999999999999</v>
-      </c>
-      <c r="H73" s="3">
-        <v>78.900000000000006</v>
-      </c>
-      <c r="I73" s="3">
-        <v>43.5</v>
-      </c>
-      <c r="J73" s="3">
-        <v>175</v>
-      </c>
-      <c r="K73" s="3">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A74" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B74" s="3">
-        <v>103</v>
-      </c>
-      <c r="C74" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E74" s="4">
-        <v>40553</v>
-      </c>
-      <c r="F74" s="4">
-        <v>45698</v>
-      </c>
-      <c r="G74" s="3">
-        <v>162</v>
-      </c>
-      <c r="H74" s="3">
-        <v>83</v>
-      </c>
-      <c r="I74" s="3">
-        <v>52</v>
-      </c>
-      <c r="J74" s="3">
+      <c r="G79">
+        <v>166</v>
+      </c>
+      <c r="H79">
+        <v>85</v>
+      </c>
+      <c r="I79">
+        <v>55.5</v>
+      </c>
+      <c r="J79">
         <v>182</v>
       </c>
-      <c r="K74" s="3">
+      <c r="K79">
         <v>170</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B75" s="3">
-        <v>103</v>
-      </c>
-      <c r="C75" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D75" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E75" s="4">
-        <v>40553</v>
-      </c>
-      <c r="F75" s="4">
-        <v>45762</v>
-      </c>
-      <c r="G75" s="3">
-        <v>162.80000000000001</v>
-      </c>
-      <c r="H75" s="3">
-        <v>83.4</v>
-      </c>
-      <c r="I75" s="3">
-        <v>52.7</v>
-      </c>
-      <c r="J75" s="3">
-        <v>182</v>
-      </c>
-      <c r="K75" s="3">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B76" s="3">
-        <v>103</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E76" s="4">
-        <v>40553</v>
-      </c>
-      <c r="F76" s="4">
-        <v>45828</v>
-      </c>
-      <c r="G76" s="3">
-        <v>163.6</v>
-      </c>
-      <c r="H76" s="3">
-        <v>83.8</v>
-      </c>
-      <c r="I76" s="3">
-        <v>53.4</v>
-      </c>
-      <c r="J76" s="3">
-        <v>182</v>
-      </c>
-      <c r="K76" s="3">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B77" s="3">
-        <v>103</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E77" s="4">
-        <v>40553</v>
-      </c>
-      <c r="F77" s="4">
-        <v>45894</v>
-      </c>
-      <c r="G77" s="3">
-        <v>164.4</v>
-      </c>
-      <c r="H77" s="3">
-        <v>84.2</v>
-      </c>
-      <c r="I77" s="3">
-        <v>54.1</v>
-      </c>
-      <c r="J77" s="3">
-        <v>182</v>
-      </c>
-      <c r="K77" s="3">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B78" s="3">
-        <v>103</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E78" s="4">
-        <v>40553</v>
-      </c>
-      <c r="F78" s="4">
-        <v>45960</v>
-      </c>
-      <c r="G78" s="3">
-        <v>165.2</v>
-      </c>
-      <c r="H78" s="3">
-        <v>84.6</v>
-      </c>
-      <c r="I78" s="3">
-        <v>54.8</v>
-      </c>
-      <c r="J78" s="3">
-        <v>182</v>
-      </c>
-      <c r="K78" s="3">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B79" s="3">
-        <v>103</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E79" s="4">
-        <v>40553</v>
-      </c>
-      <c r="F79" s="4">
-        <v>46006</v>
-      </c>
-      <c r="G79" s="3">
-        <v>166</v>
-      </c>
-      <c r="H79" s="3">
-        <v>85</v>
-      </c>
-      <c r="I79" s="3">
-        <v>55.5</v>
-      </c>
-      <c r="J79" s="3">
-        <v>182</v>
-      </c>
-      <c r="K79" s="3">
-        <v>170</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Excel with Anna instead of Ana
</commit_message>
<xml_diff>
--- a/Plantilla_Crecimiento_y_Maduracion.xlsx
+++ b/Plantilla_Crecimiento_y_Maduracion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dany\cloudestreamlit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D8F0171-D726-4D65-A091-3C7C4674DDE6}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8301CA99-4C88-45B9-9F93-2F31586BE4FC}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3204" yWindow="2388" windowWidth="16488" windowHeight="9852" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>Talento</t>
-  </si>
-  <si>
-    <t>Ana Lopez</t>
   </si>
   <si>
     <t>Gimnasia</t>
@@ -119,6 +116,9 @@
   </si>
   <si>
     <t>Fútbol</t>
+  </si>
+  <si>
+    <t>Anna Lopez</t>
   </si>
 </sst>
 </file>
@@ -717,7 +717,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="B8">
         <v>10101001</v>
@@ -726,7 +726,7 @@
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E8">
         <v>41039</v>
@@ -752,7 +752,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="B9">
         <v>10101001</v>
@@ -761,7 +761,7 @@
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E9">
         <v>41039</v>
@@ -787,7 +787,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="B10">
         <v>10101001</v>
@@ -796,7 +796,7 @@
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E10">
         <v>41039</v>
@@ -822,7 +822,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="B11">
         <v>10101001</v>
@@ -831,7 +831,7 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E11">
         <v>41039</v>
@@ -857,7 +857,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="B12">
         <v>10101001</v>
@@ -866,7 +866,7 @@
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E12">
         <v>41039</v>
@@ -892,7 +892,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="B13">
         <v>10101001</v>
@@ -901,7 +901,7 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13">
         <v>41039</v>
@@ -927,7 +927,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14">
         <v>10101002</v>
@@ -936,7 +936,7 @@
         <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E14">
         <v>40777</v>
@@ -962,7 +962,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15">
         <v>10101002</v>
@@ -971,7 +971,7 @@
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E15">
         <v>40777</v>
@@ -997,7 +997,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16">
         <v>10101002</v>
@@ -1006,7 +1006,7 @@
         <v>12</v>
       </c>
       <c r="D16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E16">
         <v>40777</v>
@@ -1032,7 +1032,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17">
         <v>10101002</v>
@@ -1041,7 +1041,7 @@
         <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E17">
         <v>40777</v>
@@ -1067,7 +1067,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18">
         <v>10101002</v>
@@ -1076,7 +1076,7 @@
         <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E18">
         <v>40777</v>
@@ -1102,7 +1102,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19">
         <v>10101002</v>
@@ -1111,7 +1111,7 @@
         <v>12</v>
       </c>
       <c r="D19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E19">
         <v>40777</v>
@@ -1137,7 +1137,7 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20">
         <v>10101003</v>
@@ -1146,7 +1146,7 @@
         <v>12</v>
       </c>
       <c r="D20" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E20">
         <v>41320</v>
@@ -1172,7 +1172,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21">
         <v>10101003</v>
@@ -1181,7 +1181,7 @@
         <v>12</v>
       </c>
       <c r="D21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E21">
         <v>41320</v>
@@ -1207,7 +1207,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B22">
         <v>10101003</v>
@@ -1216,7 +1216,7 @@
         <v>12</v>
       </c>
       <c r="D22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E22">
         <v>41320</v>
@@ -1242,7 +1242,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B23">
         <v>10101003</v>
@@ -1251,7 +1251,7 @@
         <v>12</v>
       </c>
       <c r="D23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E23">
         <v>41320</v>
@@ -1277,7 +1277,7 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B24">
         <v>10101003</v>
@@ -1286,7 +1286,7 @@
         <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E24">
         <v>41320</v>
@@ -1312,7 +1312,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B25">
         <v>10101003</v>
@@ -1321,7 +1321,7 @@
         <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E25">
         <v>41320</v>
@@ -1347,7 +1347,7 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B26">
         <v>10101004</v>
@@ -1356,7 +1356,7 @@
         <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E26">
         <v>40571</v>
@@ -1382,7 +1382,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B27">
         <v>10101004</v>
@@ -1391,7 +1391,7 @@
         <v>12</v>
       </c>
       <c r="D27" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E27">
         <v>40571</v>
@@ -1417,7 +1417,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B28">
         <v>10101004</v>
@@ -1426,7 +1426,7 @@
         <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E28">
         <v>40571</v>
@@ -1452,7 +1452,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B29">
         <v>10101004</v>
@@ -1461,7 +1461,7 @@
         <v>12</v>
       </c>
       <c r="D29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E29">
         <v>40571</v>
@@ -1487,7 +1487,7 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30">
         <v>10101004</v>
@@ -1496,7 +1496,7 @@
         <v>12</v>
       </c>
       <c r="D30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E30">
         <v>40571</v>
@@ -1522,7 +1522,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B31">
         <v>10101004</v>
@@ -1531,7 +1531,7 @@
         <v>12</v>
       </c>
       <c r="D31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E31">
         <v>40571</v>
@@ -1557,7 +1557,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32">
         <v>10101005</v>
@@ -1566,7 +1566,7 @@
         <v>12</v>
       </c>
       <c r="D32" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E32">
         <v>41548</v>
@@ -1592,7 +1592,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B33">
         <v>10101005</v>
@@ -1601,7 +1601,7 @@
         <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E33">
         <v>41548</v>
@@ -1627,7 +1627,7 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B34">
         <v>10101005</v>
@@ -1636,7 +1636,7 @@
         <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E34">
         <v>41548</v>
@@ -1662,7 +1662,7 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B35">
         <v>10101005</v>
@@ -1671,7 +1671,7 @@
         <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E35">
         <v>41548</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B36">
         <v>10101005</v>
@@ -1706,7 +1706,7 @@
         <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E36">
         <v>41548</v>
@@ -1732,7 +1732,7 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B37">
         <v>10101005</v>
@@ -1741,7 +1741,7 @@
         <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E37">
         <v>41548</v>
@@ -1767,16 +1767,16 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B38">
         <v>20202001</v>
       </c>
       <c r="C38" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D38" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E38">
         <v>40867</v>
@@ -1802,16 +1802,16 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B39">
         <v>20202001</v>
       </c>
       <c r="C39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D39" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E39">
         <v>40867</v>
@@ -1837,16 +1837,16 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B40">
         <v>20202001</v>
       </c>
       <c r="C40" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D40" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E40">
         <v>40867</v>
@@ -1872,16 +1872,16 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B41">
         <v>20202001</v>
       </c>
       <c r="C41" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D41" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E41">
         <v>40867</v>
@@ -1907,16 +1907,16 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B42">
         <v>20202001</v>
       </c>
       <c r="C42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D42" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E42">
         <v>40867</v>
@@ -1942,16 +1942,16 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B43">
         <v>20202001</v>
       </c>
       <c r="C43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D43" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E43">
         <v>40867</v>
@@ -1977,16 +1977,16 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B44">
         <v>20202002</v>
       </c>
       <c r="C44" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D44" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E44">
         <v>40426</v>
@@ -2012,16 +2012,16 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B45">
         <v>20202002</v>
       </c>
       <c r="C45" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D45" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E45">
         <v>40426</v>
@@ -2047,16 +2047,16 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B46">
         <v>20202002</v>
       </c>
       <c r="C46" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D46" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E46">
         <v>40426</v>
@@ -2082,16 +2082,16 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B47">
         <v>20202002</v>
       </c>
       <c r="C47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D47" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E47">
         <v>40426</v>
@@ -2117,16 +2117,16 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B48">
         <v>20202002</v>
       </c>
       <c r="C48" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D48" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E48">
         <v>40426</v>
@@ -2152,16 +2152,16 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B49">
         <v>20202002</v>
       </c>
       <c r="C49" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D49" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E49">
         <v>40426</v>
@@ -2187,16 +2187,16 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B50">
         <v>20202003</v>
       </c>
       <c r="C50" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D50" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E50">
         <v>41102</v>
@@ -2222,16 +2222,16 @@
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B51">
         <v>20202003</v>
       </c>
       <c r="C51" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D51" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E51">
         <v>41102</v>
@@ -2257,16 +2257,16 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B52">
         <v>20202003</v>
       </c>
       <c r="C52" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D52" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E52">
         <v>41102</v>
@@ -2292,16 +2292,16 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B53">
         <v>20202003</v>
       </c>
       <c r="C53" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D53" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E53">
         <v>41102</v>
@@ -2327,16 +2327,16 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B54">
         <v>20202003</v>
       </c>
       <c r="C54" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D54" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E54">
         <v>41102</v>
@@ -2362,16 +2362,16 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B55">
         <v>20202003</v>
       </c>
       <c r="C55" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D55" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E55">
         <v>41102</v>
@@ -2397,16 +2397,16 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B56">
         <v>20202004</v>
       </c>
       <c r="C56" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D56" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E56">
         <v>41358</v>
@@ -2432,16 +2432,16 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B57">
         <v>20202004</v>
       </c>
       <c r="C57" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D57" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E57">
         <v>41358</v>
@@ -2467,16 +2467,16 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B58">
         <v>20202004</v>
       </c>
       <c r="C58" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D58" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E58">
         <v>41358</v>
@@ -2502,16 +2502,16 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B59">
         <v>20202004</v>
       </c>
       <c r="C59" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D59" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E59">
         <v>41358</v>
@@ -2537,16 +2537,16 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B60">
         <v>20202004</v>
       </c>
       <c r="C60" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D60" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E60">
         <v>41358</v>
@@ -2572,16 +2572,16 @@
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B61">
         <v>20202004</v>
       </c>
       <c r="C61" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D61" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E61">
         <v>41358</v>
@@ -2607,16 +2607,16 @@
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B62">
         <v>101</v>
       </c>
       <c r="C62" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D62" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E62">
         <v>41044</v>
@@ -2642,16 +2642,16 @@
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B63">
         <v>101</v>
       </c>
       <c r="C63" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D63" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E63">
         <v>41044</v>
@@ -2677,16 +2677,16 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B64">
         <v>101</v>
       </c>
       <c r="C64" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D64" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E64">
         <v>41044</v>
@@ -2712,16 +2712,16 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B65">
         <v>101</v>
       </c>
       <c r="C65" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D65" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E65">
         <v>41044</v>
@@ -2747,16 +2747,16 @@
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B66">
         <v>101</v>
       </c>
       <c r="C66" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D66" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E66">
         <v>41044</v>
@@ -2782,16 +2782,16 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B67">
         <v>101</v>
       </c>
       <c r="C67" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D67" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E67">
         <v>41044</v>
@@ -2817,7 +2817,7 @@
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B68">
         <v>102</v>
@@ -2826,7 +2826,7 @@
         <v>12</v>
       </c>
       <c r="D68" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E68">
         <v>41508</v>
@@ -2852,7 +2852,7 @@
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B69">
         <v>102</v>
@@ -2861,7 +2861,7 @@
         <v>12</v>
       </c>
       <c r="D69" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E69">
         <v>41508</v>
@@ -2887,7 +2887,7 @@
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B70">
         <v>102</v>
@@ -2896,7 +2896,7 @@
         <v>12</v>
       </c>
       <c r="D70" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E70">
         <v>41508</v>
@@ -2922,7 +2922,7 @@
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B71">
         <v>102</v>
@@ -2931,7 +2931,7 @@
         <v>12</v>
       </c>
       <c r="D71" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E71">
         <v>41508</v>
@@ -2957,7 +2957,7 @@
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B72">
         <v>102</v>
@@ -2966,7 +2966,7 @@
         <v>12</v>
       </c>
       <c r="D72" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E72">
         <v>41508</v>
@@ -2992,7 +2992,7 @@
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B73">
         <v>102</v>
@@ -3001,7 +3001,7 @@
         <v>12</v>
       </c>
       <c r="D73" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E73">
         <v>41508</v>
@@ -3027,16 +3027,16 @@
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B74">
         <v>103</v>
       </c>
       <c r="C74" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D74" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E74">
         <v>40553</v>
@@ -3062,16 +3062,16 @@
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B75">
         <v>103</v>
       </c>
       <c r="C75" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D75" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E75">
         <v>40553</v>
@@ -3097,16 +3097,16 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B76">
         <v>103</v>
       </c>
       <c r="C76" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D76" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E76">
         <v>40553</v>
@@ -3132,16 +3132,16 @@
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B77">
         <v>103</v>
       </c>
       <c r="C77" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D77" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E77">
         <v>40553</v>
@@ -3167,16 +3167,16 @@
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B78">
         <v>103</v>
       </c>
       <c r="C78" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D78" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E78">
         <v>40553</v>
@@ -3202,16 +3202,16 @@
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B79">
         <v>103</v>
       </c>
       <c r="C79" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D79" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E79">
         <v>40553</v>

</xml_diff>